<commit_message>
Commit 11/20/25 #1: 1. Avance practica 3 tema 3.
</commit_message>
<xml_diff>
--- a/TAP Tema 1/results/resumen.xlsx
+++ b/TAP Tema 1/results/resumen.xlsx
@@ -174,7 +174,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="3">
@@ -190,7 +190,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Commit 11/23/25 #1: 1. Terminacion Servicios de Usuario, Registro y Aprobacion 2. Correccion de archivos 3. Pruebas menores
</commit_message>
<xml_diff>
--- a/TAP Tema 1/results/resumen.xlsx
+++ b/TAP Tema 1/results/resumen.xlsx
@@ -174,7 +174,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="3">
@@ -182,7 +182,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="4">
@@ -190,7 +190,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="5">
@@ -198,7 +198,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="6">
@@ -230,7 +230,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Commit 11/23/25 #3 : 1. Arreglar servicios de aprobaciones: borraba el nuevo, el id del registro estaba vacio, etc.
</commit_message>
<xml_diff>
--- a/TAP Tema 1/results/resumen.xlsx
+++ b/TAP Tema 1/results/resumen.xlsx
@@ -190,7 +190,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="5">
@@ -214,7 +214,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Commit 11/28/25 #1: Detalles y subir practica 4
</commit_message>
<xml_diff>
--- a/TAP Tema 1/results/resumen.xlsx
+++ b/TAP Tema 1/results/resumen.xlsx
@@ -198,7 +198,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="6">
@@ -206,7 +206,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="7">
@@ -214,7 +214,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="8">
@@ -230,7 +230,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Commit 12/02/25 #1: Practica 5 terminada
</commit_message>
<xml_diff>
--- a/TAP Tema 1/results/resumen.xlsx
+++ b/TAP Tema 1/results/resumen.xlsx
@@ -182,7 +182,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="4">
@@ -190,7 +190,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="5">

</xml_diff>